<commit_message>
Typeset Evidence Room SKU books and thicken Monday-ready Office files.
Replace cover-stub PDFs with full Diagnostic, Starter, 217-page Professional OS, Team, Blueprint, and legal-draft books. Expand Word templates, workshop/CFO decks, and example workbooks so a purchaser can start Wave 1 without living in Markdown.

Co-authored-by: adamaziz91 <adamaziz91@gmail.com>
</commit_message>
<xml_diff>
--- a/evidence-room/03_AP_AGENT_OS_PRO/Spreadsheets/ER_AP_Agent_Registry.xlsx
+++ b/evidence-room/03_AP_AGENT_OS_PRO/Spreadsheets/ER_AP_Agent_Registry.xlsx
@@ -8,6 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AGENT_REGISTRY" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXAMPLE_NORTHLINE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BLANK_REGISTER" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCTIONS" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -82,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -91,6 +94,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1137,4 +1143,1182 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Default autonomy</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Level in force</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Human owner</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Wave</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Exclusions (hard)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Last recert</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Invoice Intake</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Elena Voss</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>shadow</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Invoice Validation</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Elena Voss</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>shadow</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Matching</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Elena Voss</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>shadow</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Exception Triage</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Exception Desk (designate)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>shadow</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Goods Receipt</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>not commissioned</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Plant liaison (designate)</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>PO Quality</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>not commissioned</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>James Okonkwo</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Approval</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>not commissioned</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Approvals coordinator (designate)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Supplier Resolution</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>not commissioned</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Supplier desk (designate)</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Internal Follow-up</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>not commissioned</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Exception Desk (designate)</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Duplicate &amp; Anomaly</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Priya Shah / Controls</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>shadow</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Vendor Statement</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>not commissioned</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliations (designate)</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Payment Proposal Review</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>not commissioned</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Hannah Reid</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Never release or transmit payment</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>AP Close</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>not commissioned</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Priya Shah</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>AP Reporting</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>not commissioned</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>AP Analytics (designate)</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Root Cause</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>not commissioned</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Transformation (designate)</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Orchestrator</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Marcus Chen</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>shadow</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Payment / vendor-bank / close attestation</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Default autonomy</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Level in force</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Human owner</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Wave</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Exclusions (hard)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Last recert</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Invoice Intake</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Invoice Validation</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Matching</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Exception Triage</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Goods Receipt</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>PO Quality</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Approval</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Supplier Resolution</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Internal Follow-up</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Duplicate &amp; Anomaly</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Vendor Statement</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Payment Proposal Review</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>AP Close</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>AP Reporting</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Root Cause</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Orchestrator</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>One row per live helper, including informal copilots. Agents cannot hold Accountable. Payment has no promotion path. Northline is fictional.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>